<commit_message>
Update สระบุรี web data 1.1.5
</commit_message>
<xml_diff>
--- a/data_สระบุรี.xlsx
+++ b/data_สระบุรี.xlsx
@@ -515,7 +515,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D233"/>
+  <dimension ref="A1:D241"/>
   <cols>
     <col min="1" max="1" width="23.53515625" customWidth="1"/>
     <col min="2" max="2" width="19.53515625" customWidth="1"/>
@@ -651,13 +651,13 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="str">
-        <v>EQPTZ2501096</v>
+        <v>EFAZZ0001862</v>
       </c>
       <c r="B10" s="5" t="str">
         <v>400G PSM4</v>
       </c>
       <c r="C10" s="6" t="str">
-        <v>#09</v>
+        <v>#11</v>
       </c>
       <c r="D10" s="5" t="str">
         <v>TRX FA</v>
@@ -665,13 +665,13 @@
     </row>
     <row r="11">
       <c r="A11" s="5" t="str">
-        <v>EFAZZ0000923</v>
+        <v>EQPTZ2501105</v>
       </c>
       <c r="B11" s="5" t="str">
         <v>400G PSM4</v>
       </c>
       <c r="C11" s="6" t="str">
-        <v>#10</v>
+        <v>#12</v>
       </c>
       <c r="D11" s="5" t="str">
         <v>TRX FA</v>
@@ -679,13 +679,13 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="str">
-        <v>EFAZZ0001862</v>
+        <v>EZDYH2400126</v>
       </c>
       <c r="B12" s="5" t="str">
         <v>400G PSM4</v>
       </c>
       <c r="C12" s="6" t="str">
-        <v>#11</v>
+        <v>#13</v>
       </c>
       <c r="D12" s="5" t="str">
         <v>TRX FA</v>
@@ -693,13 +693,13 @@
     </row>
     <row r="13">
       <c r="A13" s="5" t="str">
-        <v>EQPTZ2501105</v>
+        <v>EQPTZ2500010</v>
       </c>
       <c r="B13" s="5" t="str">
         <v>400G PSM4</v>
       </c>
       <c r="C13" s="6" t="str">
-        <v>#12</v>
+        <v>#15</v>
       </c>
       <c r="D13" s="5" t="str">
         <v>TRX FA</v>
@@ -707,13 +707,13 @@
     </row>
     <row r="14">
       <c r="A14" s="5" t="str">
-        <v>EZDYH2400126</v>
+        <v>EZDYH0000128</v>
       </c>
       <c r="B14" s="5" t="str">
         <v>400G PSM4</v>
       </c>
       <c r="C14" s="6" t="str">
-        <v>#13</v>
+        <v>#18</v>
       </c>
       <c r="D14" s="5" t="str">
         <v>TRX FA</v>
@@ -721,13 +721,13 @@
     </row>
     <row r="15">
       <c r="A15" s="5" t="str">
-        <v>EZDYH2400098</v>
+        <v>EQPTZ2500007</v>
       </c>
       <c r="B15" s="5" t="str">
         <v>400G PSM4</v>
       </c>
       <c r="C15" s="6" t="str">
-        <v>#14</v>
+        <v>#19</v>
       </c>
       <c r="D15" s="5" t="str">
         <v>TRX FA</v>
@@ -735,13 +735,13 @@
     </row>
     <row r="16">
       <c r="A16" s="5" t="str">
-        <v>EQPTZ2500010</v>
+        <v>EFAZZ0001863</v>
       </c>
       <c r="B16" s="5" t="str">
         <v>400G PSM4</v>
       </c>
       <c r="C16" s="6" t="str">
-        <v>#15</v>
+        <v>#20</v>
       </c>
       <c r="D16" s="5" t="str">
         <v>TRX FA</v>
@@ -749,13 +749,13 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="str">
-        <v>EQPTZ2501103</v>
+        <v>EFAZZ0000974</v>
       </c>
       <c r="B17" s="5" t="str">
         <v>400G PSM4</v>
       </c>
       <c r="C17" s="6" t="str">
-        <v>#16</v>
+        <v>#21</v>
       </c>
       <c r="D17" s="5" t="str">
         <v>TRX FA</v>
@@ -763,13 +763,13 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="str">
-        <v>EZDYH2400089</v>
+        <v>EFAZZ0001737</v>
       </c>
       <c r="B18" s="5" t="str">
         <v>400G PSM4</v>
       </c>
       <c r="C18" s="6" t="str">
-        <v>#17</v>
+        <v>#26</v>
       </c>
       <c r="D18" s="5" t="str">
         <v>TRX FA</v>
@@ -777,139 +777,139 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="str">
-        <v>EZDYH0000128</v>
+        <v/>
       </c>
       <c r="B19" s="5" t="str">
-        <v>400G PSM4</v>
+        <v/>
       </c>
       <c r="C19" s="6" t="str">
-        <v>#18</v>
+        <v/>
       </c>
       <c r="D19" s="5" t="str">
-        <v>TRX FA</v>
+        <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="str">
-        <v>EQPTZ2500007</v>
+        <v>EFAZZ0001615</v>
       </c>
       <c r="B20" s="5" t="str">
         <v>400G PSM4</v>
       </c>
       <c r="C20" s="6" t="str">
-        <v>#19</v>
+        <v>#01</v>
       </c>
       <c r="D20" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="str">
-        <v>EFAZZ0001863</v>
+        <v>EYHJE0000112</v>
       </c>
       <c r="B21" s="5" t="str">
         <v>400G PSM4</v>
       </c>
       <c r="C21" s="6" t="str">
-        <v>#20</v>
+        <v>#02</v>
       </c>
       <c r="D21" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="str">
-        <v>EFAZZ0000974</v>
+        <v>EYHJE2400046</v>
       </c>
       <c r="B22" s="5" t="str">
         <v>400G PSM4</v>
       </c>
       <c r="C22" s="6" t="str">
-        <v>#21</v>
+        <v>#07</v>
       </c>
       <c r="D22" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="str">
-        <v>EQPTZ2501069</v>
+        <v>EFAZZ0000853</v>
       </c>
       <c r="B23" s="5" t="str">
         <v>400G PSM4</v>
       </c>
       <c r="C23" s="6" t="str">
-        <v>#22</v>
+        <v>#11</v>
       </c>
       <c r="D23" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="str">
-        <v>EZDYH2400101</v>
+        <v>EFAZZ0000859</v>
       </c>
       <c r="B24" s="5" t="str">
         <v>400G PSM4</v>
       </c>
       <c r="C24" s="6" t="str">
-        <v>#23</v>
+        <v>#12</v>
       </c>
       <c r="D24" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="str">
-        <v>EZDYH2400102</v>
+        <v>EFAZZ0000845</v>
       </c>
       <c r="B25" s="5" t="str">
         <v>400G PSM4</v>
       </c>
       <c r="C25" s="6" t="str">
-        <v>#24</v>
+        <v>#13</v>
       </c>
       <c r="D25" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="str">
-        <v>EQPTZ2501082</v>
+        <v>EFAZZ0001035</v>
       </c>
       <c r="B26" s="5" t="str">
         <v>400G PSM4</v>
       </c>
       <c r="C26" s="6" t="str">
-        <v>#25</v>
+        <v>#13</v>
       </c>
       <c r="D26" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="str">
-        <v/>
+        <v>EFAZZ0000283</v>
       </c>
       <c r="B27" s="5" t="str">
-        <v/>
+        <v>400G PSM4</v>
       </c>
       <c r="C27" s="6" t="str">
-        <v/>
+        <v>#14</v>
       </c>
       <c r="D27" s="5" t="str">
-        <v/>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="str">
-        <v>EFAZZ0001615</v>
+        <v>EYHJE2400027</v>
       </c>
       <c r="B28" s="5" t="str">
         <v>400G PSM4</v>
       </c>
       <c r="C28" s="6" t="str">
-        <v>#01</v>
+        <v>#15</v>
       </c>
       <c r="D28" s="5" t="str">
         <v>TX AA</v>
@@ -917,13 +917,13 @@
     </row>
     <row r="29">
       <c r="A29" s="5" t="str">
-        <v>EYHJE0000112</v>
+        <v>EFAZZ0001038</v>
       </c>
       <c r="B29" s="5" t="str">
         <v>400G PSM4</v>
       </c>
       <c r="C29" s="6" t="str">
-        <v>#02</v>
+        <v>#16</v>
       </c>
       <c r="D29" s="5" t="str">
         <v>TX AA</v>
@@ -931,13 +931,13 @@
     </row>
     <row r="30">
       <c r="A30" s="5" t="str">
-        <v>EFAZZ0001603</v>
+        <v>EFAZZ0000815</v>
       </c>
       <c r="B30" s="5" t="str">
         <v>400G PSM4</v>
       </c>
       <c r="C30" s="6" t="str">
-        <v>#03</v>
+        <v>#17</v>
       </c>
       <c r="D30" s="5" t="str">
         <v>TX AA</v>
@@ -945,13 +945,13 @@
     </row>
     <row r="31">
       <c r="A31" s="5" t="str">
-        <v>EFAZZ0001041</v>
+        <v>EFAZZ0001601</v>
       </c>
       <c r="B31" s="5" t="str">
         <v>400G PSM4</v>
       </c>
       <c r="C31" s="6" t="str">
-        <v>#04</v>
+        <v>#19</v>
       </c>
       <c r="D31" s="5" t="str">
         <v>TX AA</v>
@@ -959,13 +959,13 @@
     </row>
     <row r="32">
       <c r="A32" s="5" t="str">
-        <v>EFAZZ0001604</v>
+        <v>EYHJE2400029</v>
       </c>
       <c r="B32" s="5" t="str">
         <v>400G PSM4</v>
       </c>
       <c r="C32" s="6" t="str">
-        <v>#05</v>
+        <v>#20</v>
       </c>
       <c r="D32" s="5" t="str">
         <v>TX AA</v>
@@ -973,13 +973,13 @@
     </row>
     <row r="33">
       <c r="A33" s="5" t="str">
-        <v>EFAZZ0001733</v>
+        <v>EFAZZ0001735</v>
       </c>
       <c r="B33" s="5" t="str">
         <v>400G PSM4</v>
       </c>
       <c r="C33" s="6" t="str">
-        <v>#06</v>
+        <v>#21</v>
       </c>
       <c r="D33" s="5" t="str">
         <v>TX AA</v>
@@ -987,321 +987,321 @@
     </row>
     <row r="34">
       <c r="A34" s="5" t="str">
-        <v>EYHJE2400046</v>
+        <v/>
       </c>
       <c r="B34" s="5" t="str">
-        <v>400G PSM4</v>
+        <v/>
       </c>
       <c r="C34" s="6" t="str">
-        <v>#07</v>
+        <v/>
       </c>
       <c r="D34" s="5" t="str">
-        <v>TX AA</v>
+        <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="str">
-        <v>EFAZZ0001599</v>
+        <v>EQPTZ2501069</v>
       </c>
       <c r="B35" s="5" t="str">
-        <v>400G PSM4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C35" s="6" t="str">
-        <v>#08</v>
+        <v>#02</v>
       </c>
       <c r="D35" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="str">
-        <v>EFAZZ0001730</v>
+        <v>EQPTZ2501082</v>
       </c>
       <c r="B36" s="5" t="str">
-        <v>400G PSM4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C36" s="6" t="str">
-        <v>#09</v>
+        <v>#03</v>
       </c>
       <c r="D36" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="str">
-        <v>EFAZZ0000868</v>
+        <v>EZDYH2400101</v>
       </c>
       <c r="B37" s="5" t="str">
-        <v>400G PSM4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C37" s="6" t="str">
-        <v>#10</v>
+        <v>#04</v>
       </c>
       <c r="D37" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="str">
-        <v>EFAZZ0000853</v>
+        <v>EZDYH2400102</v>
       </c>
       <c r="B38" s="5" t="str">
-        <v>400G PSM4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C38" s="6" t="str">
-        <v>#11</v>
+        <v>#05</v>
       </c>
       <c r="D38" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="str">
-        <v>EFAZZ0000859</v>
+        <v>EZDYH2400132</v>
       </c>
       <c r="B39" s="5" t="str">
-        <v>400G PSM4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C39" s="6" t="str">
-        <v>#12</v>
+        <v>#06</v>
       </c>
       <c r="D39" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="str">
-        <v>EFAZZ0000845</v>
+        <v>EZDYH2400118</v>
       </c>
       <c r="B40" s="5" t="str">
-        <v>400G PSM4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C40" s="6" t="str">
-        <v>#13</v>
+        <v>#07</v>
       </c>
       <c r="D40" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="str">
-        <v>EFAZZ0001035</v>
+        <v>EQPTZ2501098</v>
       </c>
       <c r="B41" s="5" t="str">
-        <v>400G PSM4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C41" s="6" t="str">
-        <v>#13</v>
+        <v>#08</v>
       </c>
       <c r="D41" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="str">
-        <v>EFAZZ0000283</v>
+        <v>EQPTZ2501096</v>
       </c>
       <c r="B42" s="5" t="str">
-        <v>400G PSM4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C42" s="6" t="str">
-        <v>#14</v>
+        <v>#09</v>
       </c>
       <c r="D42" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="str">
-        <v>EYHJE2400027</v>
+        <v>EFAZZ0000923</v>
       </c>
       <c r="B43" s="5" t="str">
-        <v>400G PSM4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C43" s="6" t="str">
-        <v>#15</v>
+        <v>#10</v>
       </c>
       <c r="D43" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="str">
-        <v>EFAZZ0001038</v>
+        <v>EQPTZ2501103</v>
       </c>
       <c r="B44" s="5" t="str">
-        <v>400G PSM4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C44" s="6" t="str">
-        <v>#16</v>
+        <v>#11</v>
       </c>
       <c r="D44" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="str">
-        <v>EFAZZ0000815</v>
+        <v>EQPTZ2501072</v>
       </c>
       <c r="B45" s="5" t="str">
-        <v>400G PSM4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C45" s="6" t="str">
-        <v>#17</v>
+        <v>#14</v>
       </c>
       <c r="D45" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="str">
-        <v>EFAZZ0000816</v>
+        <v>EQPTZ2501074</v>
       </c>
       <c r="B46" s="5" t="str">
-        <v>400G PSM4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C46" s="6" t="str">
-        <v>#18</v>
+        <v>#15</v>
       </c>
       <c r="D46" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="str">
-        <v>EFAZZ0001601</v>
+        <v>EQPTZ2501065</v>
       </c>
       <c r="B47" s="5" t="str">
-        <v>400G PSM4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C47" s="6" t="str">
-        <v>#19</v>
+        <v>#16</v>
       </c>
       <c r="D47" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="str">
-        <v>EYHJE2400029</v>
+        <v>EQPTZ2501095</v>
       </c>
       <c r="B48" s="5" t="str">
-        <v>400G PSM4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C48" s="6" t="str">
-        <v>#20</v>
+        <v>#18</v>
       </c>
       <c r="D48" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="str">
-        <v>EFAZZ0001735</v>
+        <v>EQPTZ2501064</v>
       </c>
       <c r="B49" s="5" t="str">
-        <v>400G PSM4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C49" s="6" t="str">
-        <v>#21</v>
+        <v>#19</v>
       </c>
       <c r="D49" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="str">
-        <v/>
+        <v>EQPTZ2501066</v>
       </c>
       <c r="B50" s="5" t="str">
-        <v/>
+        <v>800G DR8</v>
       </c>
       <c r="C50" s="6" t="str">
-        <v/>
+        <v>#20</v>
       </c>
       <c r="D50" s="5" t="str">
-        <v/>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="str">
-        <v>EFAZZ0001559</v>
+        <v>EFAZZ0000975</v>
       </c>
       <c r="B51" s="5" t="str">
-        <v>200G AOC GEN2</v>
+        <v>800G DR8</v>
       </c>
       <c r="C51" s="6" t="str">
-        <v>#00</v>
+        <v>#21</v>
       </c>
       <c r="D51" s="5" t="str">
-        <v>MM AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="str">
-        <v>EZDYH0000111</v>
+        <v>EFAZZ0000973</v>
       </c>
       <c r="B52" s="5" t="str">
-        <v>200G AOC GEN2</v>
+        <v>800G DR8</v>
       </c>
       <c r="C52" s="6" t="str">
-        <v>#00</v>
+        <v>#22</v>
       </c>
       <c r="D52" s="5" t="str">
-        <v>MM AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="str">
-        <v/>
+        <v>EFAZZ0000972</v>
       </c>
       <c r="B53" s="5" t="str">
-        <v/>
+        <v>800G DR8</v>
       </c>
       <c r="C53" s="6" t="str">
-        <v/>
+        <v>#23</v>
       </c>
       <c r="D53" s="5" t="str">
-        <v/>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="str">
-        <v>EFAZZ0000820</v>
+        <v>EFAZZ0001007</v>
       </c>
       <c r="B54" s="5" t="str">
-        <v>400G CGR4+</v>
+        <v>800G DR8</v>
       </c>
       <c r="C54" s="6" t="str">
-        <v>#05</v>
+        <v>#24</v>
       </c>
       <c r="D54" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="str">
-        <v>EFAZZ0000851</v>
+        <v/>
       </c>
       <c r="B55" s="5" t="str">
-        <v>400G CGR4+</v>
+        <v/>
       </c>
       <c r="C55" s="6" t="str">
-        <v>#06</v>
+        <v/>
       </c>
       <c r="D55" s="5" t="str">
-        <v>TX AA</v>
+        <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="str">
-        <v>EZDYH0000057</v>
+        <v>EFAZZ0001603</v>
       </c>
       <c r="B56" s="5" t="str">
-        <v>400G CGR4+</v>
+        <v>800G DR8</v>
       </c>
       <c r="C56" s="6" t="str">
-        <v>#08</v>
+        <v>#01</v>
       </c>
       <c r="D56" s="5" t="str">
         <v>TX AA</v>
@@ -1309,13 +1309,13 @@
     </row>
     <row r="57">
       <c r="A57" s="5" t="str">
-        <v>EZDYH0000066</v>
+        <v>EQPTZ2501075</v>
       </c>
       <c r="B57" s="5" t="str">
-        <v>400G CGR4+</v>
+        <v>800G DR8</v>
       </c>
       <c r="C57" s="6" t="str">
-        <v>#09</v>
+        <v>#02</v>
       </c>
       <c r="D57" s="5" t="str">
         <v>TX AA</v>
@@ -1323,293 +1323,293 @@
     </row>
     <row r="58">
       <c r="A58" s="5" t="str">
-        <v/>
+        <v>EQPTZ2501076</v>
       </c>
       <c r="B58" s="5" t="str">
-        <v/>
+        <v>800G DR8</v>
       </c>
       <c r="C58" s="6" t="str">
-        <v/>
+        <v>#03</v>
       </c>
       <c r="D58" s="5" t="str">
-        <v/>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="str">
-        <v>EFAZZ0001006</v>
+        <v>EFAZZ0001041</v>
       </c>
       <c r="B59" s="5" t="str">
-        <v>400G DR4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C59" s="6" t="str">
-        <v>#15</v>
+        <v>#04</v>
       </c>
       <c r="D59" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="str">
-        <v>EFAZZ0001005</v>
+        <v>EFAZZ0001604</v>
       </c>
       <c r="B60" s="5" t="str">
-        <v>400G DR4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C60" s="6" t="str">
-        <v>#16</v>
+        <v>#05</v>
       </c>
       <c r="D60" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="str">
-        <v>EFAZZ0000282</v>
+        <v>EFAZZ0001733</v>
       </c>
       <c r="B61" s="5" t="str">
-        <v>400G DR4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C61" s="6" t="str">
-        <v>#18</v>
+        <v>#06</v>
       </c>
       <c r="D61" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="str">
-        <v>EFAZZ0000924</v>
+        <v>EQPTZ2501086</v>
       </c>
       <c r="B62" s="5" t="str">
-        <v>400G DR4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C62" s="6" t="str">
-        <v>#19</v>
+        <v>#07</v>
       </c>
       <c r="D62" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="str">
-        <v>EFAZZ0001737</v>
+        <v>EQPTZ2501085</v>
       </c>
       <c r="B63" s="5" t="str">
-        <v>400G DR4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C63" s="6" t="str">
-        <v>#25</v>
+        <v>#08</v>
       </c>
       <c r="D63" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="str">
-        <v>EFAZZ0001042</v>
+        <v>EFAZZ0001599</v>
       </c>
       <c r="B64" s="5" t="str">
-        <v>400G DR4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C64" s="6" t="str">
-        <v>#26</v>
+        <v>#09</v>
       </c>
       <c r="D64" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="str">
-        <v>EFAZZ0001043</v>
+        <v>EFAZZ0001730</v>
       </c>
       <c r="B65" s="5" t="str">
-        <v>400G DR4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C65" s="6" t="str">
-        <v>#27</v>
+        <v>#10</v>
       </c>
       <c r="D65" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="str">
-        <v>EFAZZ0001045</v>
+        <v>EQPTZ2501087</v>
       </c>
       <c r="B66" s="5" t="str">
-        <v>400G DR4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C66" s="6" t="str">
-        <v>#28</v>
+        <v>#11</v>
       </c>
       <c r="D66" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="str">
-        <v>EFAZZ0001044</v>
+        <v>EQPTZ2501091</v>
       </c>
       <c r="B67" s="5" t="str">
-        <v>400G DR4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C67" s="6" t="str">
-        <v>#29</v>
+        <v>#12</v>
       </c>
       <c r="D67" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="str">
-        <v>EFAZZ0000922</v>
+        <v>EQPTZ2501090</v>
       </c>
       <c r="B68" s="5" t="str">
-        <v>400G DR4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C68" s="6" t="str">
-        <v>#37</v>
+        <v>#13</v>
       </c>
       <c r="D68" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="str">
-        <v>EFAZZ0001849</v>
+        <v>EZDYH2400213</v>
       </c>
       <c r="B69" s="5" t="str">
-        <v>400G DR4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C69" s="6" t="str">
-        <v>#48</v>
+        <v>#18</v>
       </c>
       <c r="D69" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="str">
-        <v>EFAZZ0001856</v>
+        <v>EFAZZ0001607</v>
       </c>
       <c r="B70" s="5" t="str">
-        <v>400G DR4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C70" s="6" t="str">
-        <v>#49</v>
+        <v>#22</v>
       </c>
       <c r="D70" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="str">
-        <v>EFAZZ0001855</v>
+        <v>EFAZZ0001605</v>
       </c>
       <c r="B71" s="5" t="str">
-        <v>400G DR4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C71" s="6" t="str">
-        <v>#51</v>
+        <v>#23</v>
       </c>
       <c r="D71" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="str">
-        <v>EFAZZ0001848</v>
+        <v>EFAZZ0001608</v>
       </c>
       <c r="B72" s="5" t="str">
-        <v>400G DR4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C72" s="6" t="str">
-        <v>#52</v>
+        <v>#24</v>
       </c>
       <c r="D72" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="str">
-        <v>EFAZZ0001847</v>
+        <v>EYHJE2400044</v>
       </c>
       <c r="B73" s="5" t="str">
-        <v>400G DR4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C73" s="6" t="str">
-        <v>#53</v>
+        <v>#25</v>
       </c>
       <c r="D73" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="str">
-        <v>EFAZZ0001846</v>
+        <v>EFAZZ0001606</v>
       </c>
       <c r="B74" s="5" t="str">
-        <v>400G DR4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C74" s="6" t="str">
-        <v>#54</v>
+        <v>#26</v>
       </c>
       <c r="D74" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="str">
-        <v>EFAZZ0000842</v>
+        <v>EYHJE2400018</v>
       </c>
       <c r="B75" s="5" t="str">
-        <v>400G DR4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C75" s="6" t="str">
-        <v>#55</v>
+        <v>#27</v>
       </c>
       <c r="D75" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="5" t="str">
-        <v>EFAZZ0001845</v>
+        <v>EFAZZ0001625</v>
       </c>
       <c r="B76" s="5" t="str">
-        <v>400G DR4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C76" s="6" t="str">
-        <v>#56</v>
+        <v>#28</v>
       </c>
       <c r="D76" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="5" t="str">
-        <v/>
+        <v>EYHJE2400028</v>
       </c>
       <c r="B77" s="5" t="str">
-        <v/>
+        <v>800G DR8</v>
       </c>
       <c r="C77" s="6" t="str">
-        <v/>
+        <v>#29</v>
       </c>
       <c r="D77" s="5" t="str">
-        <v/>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="5" t="str">
-        <v>EFAZZ0001605</v>
+        <v>EFAZZ0000854</v>
       </c>
       <c r="B78" s="5" t="str">
-        <v>400G DR4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C78" s="6" t="str">
-        <v>#09</v>
+        <v>#30</v>
       </c>
       <c r="D78" s="5" t="str">
         <v>TX AA</v>
@@ -1617,13 +1617,13 @@
     </row>
     <row r="79">
       <c r="A79" s="5" t="str">
-        <v>EFAZZ0001646</v>
+        <v>EFAZZ0000852</v>
       </c>
       <c r="B79" s="5" t="str">
-        <v>400G DR4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C79" s="6" t="str">
-        <v>#35</v>
+        <v>#31</v>
       </c>
       <c r="D79" s="5" t="str">
         <v>TX AA</v>
@@ -1631,13 +1631,13 @@
     </row>
     <row r="80">
       <c r="A80" s="5" t="str">
-        <v>EFAZZ0001565</v>
+        <v>EFAZZ0001734</v>
       </c>
       <c r="B80" s="5" t="str">
-        <v>400G DR4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C80" s="6" t="str">
-        <v>#36</v>
+        <v>#32</v>
       </c>
       <c r="D80" s="5" t="str">
         <v>TX AA</v>
@@ -1645,13 +1645,13 @@
     </row>
     <row r="81">
       <c r="A81" s="5" t="str">
-        <v>EFAZZ0001600</v>
+        <v>EFAZZ0001566</v>
       </c>
       <c r="B81" s="5" t="str">
-        <v>400G DR4</v>
+        <v>800G DR8</v>
       </c>
       <c r="C81" s="6" t="str">
-        <v>#37</v>
+        <v>#33</v>
       </c>
       <c r="D81" s="5" t="str">
         <v>TX AA</v>
@@ -1659,58 +1659,58 @@
     </row>
     <row r="82">
       <c r="A82" s="5" t="str">
-        <v>EFAZZ0001602</v>
+        <v/>
       </c>
       <c r="B82" s="5" t="str">
-        <v>400G DR4</v>
+        <v/>
       </c>
       <c r="C82" s="6" t="str">
-        <v>#38</v>
+        <v/>
       </c>
       <c r="D82" s="5" t="str">
-        <v>TX AA</v>
+        <v/>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="str">
-        <v>EFAZZ0001566</v>
+        <v>EFAZZ2400191</v>
       </c>
       <c r="B83" s="5" t="str">
-        <v>400G DR4</v>
+        <v>800G DR8 AWS</v>
       </c>
       <c r="C83" s="6" t="str">
-        <v>#46</v>
+        <v>#01</v>
       </c>
       <c r="D83" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="str">
-        <v>EFAZZ0001625</v>
+        <v>EZDYH2400192</v>
       </c>
       <c r="B84" s="5" t="str">
-        <v>400G DR4</v>
+        <v>800G DR8 AWS</v>
       </c>
       <c r="C84" s="6" t="str">
-        <v>#47</v>
+        <v>#02</v>
       </c>
       <c r="D84" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="str">
-        <v>EYHJE2400028</v>
+        <v>EZDYH2400098</v>
       </c>
       <c r="B85" s="5" t="str">
-        <v>400G DR4</v>
+        <v>800G DR8 AWS</v>
       </c>
       <c r="C85" s="6" t="str">
-        <v>#48</v>
+        <v>#03</v>
       </c>
       <c r="D85" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="86">
@@ -1729,44 +1729,44 @@
     </row>
     <row r="87">
       <c r="A87" s="5" t="str">
-        <v>EYHJE2400025</v>
+        <v>EZDYH2400055</v>
       </c>
       <c r="B87" s="5" t="str">
-        <v>800G 2XFR4 GEN1</v>
+        <v>800G DR8 AWS</v>
       </c>
       <c r="C87" s="6" t="str">
         <v>#01</v>
       </c>
       <c r="D87" s="5" t="str">
-        <v>TX AA  [ NPI ]</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="5" t="str">
-        <v/>
+        <v>EQPTZ2501083</v>
       </c>
       <c r="B88" s="5" t="str">
-        <v/>
+        <v>800G DR8 AWS</v>
       </c>
       <c r="C88" s="6" t="str">
-        <v/>
+        <v>#02</v>
       </c>
       <c r="D88" s="5" t="str">
-        <v/>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="5" t="str">
-        <v>EFAZZ0001772</v>
+        <v>EQPTZ2501101</v>
       </c>
       <c r="B89" s="5" t="str">
-        <v>800G 2XFR4 GEN1</v>
+        <v>800G DR8 AWS</v>
       </c>
       <c r="C89" s="6" t="str">
-        <v>#02</v>
+        <v>#06</v>
       </c>
       <c r="D89" s="5" t="str">
-        <v>TX AA [ NPI ]</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="90">
@@ -1785,223 +1785,223 @@
     </row>
     <row r="91">
       <c r="A91" s="5" t="str">
-        <v>EQPTZ2400147</v>
+        <v>EZDYH2400089</v>
       </c>
       <c r="B91" s="5" t="str">
-        <v>800G DR8</v>
+        <v>400G DR4 GEN1</v>
       </c>
       <c r="C91" s="6" t="str">
         <v>#01</v>
       </c>
       <c r="D91" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TRX FA [ NPI ]</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="5" t="str">
-        <v>EQPTZ2501078</v>
+        <v/>
       </c>
       <c r="B92" s="5" t="str">
-        <v>800G DR8</v>
+        <v/>
       </c>
       <c r="C92" s="6" t="str">
-        <v>#03</v>
+        <v/>
       </c>
       <c r="D92" s="5" t="str">
-        <v>TRX FA</v>
+        <v/>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="5" t="str">
-        <v>EZDYH2400132</v>
+        <v>EFAZZ0001602</v>
       </c>
       <c r="B93" s="5" t="str">
-        <v>800G DR8</v>
+        <v>400G DR4 GEN1</v>
       </c>
       <c r="C93" s="6" t="str">
-        <v>#06</v>
+        <v>#01</v>
       </c>
       <c r="D93" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA [ NPI ]</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="5" t="str">
-        <v>EZDYH2400118</v>
+        <v/>
       </c>
       <c r="B94" s="5" t="str">
-        <v>800G DR8</v>
+        <v/>
       </c>
       <c r="C94" s="6" t="str">
-        <v>#07</v>
+        <v/>
       </c>
       <c r="D94" s="5" t="str">
-        <v>TRX FA</v>
+        <v/>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="5" t="str">
-        <v>EQPTZ2501072</v>
+        <v>EFAZZ2400673</v>
       </c>
       <c r="B95" s="5" t="str">
-        <v>800G DR8</v>
+        <v>800G 2XFR4</v>
       </c>
       <c r="C95" s="6" t="str">
-        <v>#14</v>
+        <v>#01</v>
       </c>
       <c r="D95" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="5" t="str">
-        <v>EQPTZ2501074</v>
+        <v>EQPTZ2500004</v>
       </c>
       <c r="B96" s="5" t="str">
-        <v>800G DR8</v>
+        <v>800G 2XFR4</v>
       </c>
       <c r="C96" s="6" t="str">
-        <v>#15</v>
+        <v>#02</v>
       </c>
       <c r="D96" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="5" t="str">
-        <v>EQPTZ2501065</v>
+        <v>EQPTZ2500005</v>
       </c>
       <c r="B97" s="5" t="str">
-        <v>800G DR8</v>
+        <v>800G 2XFR4</v>
       </c>
       <c r="C97" s="6" t="str">
-        <v>#16</v>
+        <v>#03</v>
       </c>
       <c r="D97" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="5" t="str">
-        <v>EQPTZ2501095</v>
+        <v>EZDYH2400051</v>
       </c>
       <c r="B98" s="5" t="str">
-        <v>800G DR8</v>
+        <v>800G 2XFR4</v>
       </c>
       <c r="C98" s="6" t="str">
-        <v>#18</v>
+        <v>#04</v>
       </c>
       <c r="D98" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="5" t="str">
-        <v>EQPTZ2501064</v>
+        <v>EQPTZ2400292</v>
       </c>
       <c r="B99" s="5" t="str">
-        <v>800G DR8</v>
+        <v>800G 2XFR4</v>
       </c>
       <c r="C99" s="6" t="str">
-        <v>#19</v>
+        <v>#05</v>
       </c>
       <c r="D99" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="5" t="str">
-        <v>EQPTZ2501066</v>
+        <v>EZDYH2400088</v>
       </c>
       <c r="B100" s="5" t="str">
-        <v>800G DR8</v>
+        <v>800G 2XFR4</v>
       </c>
       <c r="C100" s="6" t="str">
-        <v>#20</v>
+        <v>#06</v>
       </c>
       <c r="D100" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="5" t="str">
-        <v>EFAZZ0000975</v>
+        <v>EZDYH2400191</v>
       </c>
       <c r="B101" s="5" t="str">
-        <v>800G DR8</v>
+        <v>800G 2XFR4</v>
       </c>
       <c r="C101" s="6" t="str">
-        <v>#21</v>
+        <v>#07</v>
       </c>
       <c r="D101" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="5" t="str">
-        <v>EFAZZ0000973</v>
+        <v>EQPTZ2501089</v>
       </c>
       <c r="B102" s="5" t="str">
-        <v>800G DR8</v>
+        <v>800G 2XFR4</v>
       </c>
       <c r="C102" s="6" t="str">
-        <v>#22</v>
+        <v>#08</v>
       </c>
       <c r="D102" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="5" t="str">
-        <v>EFAZZ0000972</v>
+        <v>EQPTZ2501093</v>
       </c>
       <c r="B103" s="5" t="str">
-        <v>800G DR8</v>
+        <v>800G 2XFR4</v>
       </c>
       <c r="C103" s="6" t="str">
-        <v>#23</v>
+        <v>#09</v>
       </c>
       <c r="D103" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="5" t="str">
-        <v>EFAZZ0001007</v>
+        <v>EQPTZ2500009</v>
       </c>
       <c r="B104" s="5" t="str">
-        <v>800G DR8</v>
+        <v>800G 2XFR4</v>
       </c>
       <c r="C104" s="6" t="str">
-        <v>#24</v>
+        <v>#10</v>
       </c>
       <c r="D104" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="5" t="str">
-        <v/>
+        <v>EQPTZ2501077</v>
       </c>
       <c r="B105" s="5" t="str">
-        <v/>
+        <v>800G 2XFR4</v>
       </c>
       <c r="C105" s="6" t="str">
-        <v/>
+        <v>#11</v>
       </c>
       <c r="D105" s="5" t="str">
-        <v/>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="5" t="str">
-        <v>EZDYH2400214</v>
+        <v>EQPTZ2501079</v>
       </c>
       <c r="B106" s="5" t="str">
-        <v>800G DR8</v>
+        <v>800G 2XFR4</v>
       </c>
       <c r="C106" s="6" t="str">
-        <v>#01</v>
+        <v>#12</v>
       </c>
       <c r="D106" s="5" t="str">
         <v>TX AA</v>
@@ -2009,13 +2009,13 @@
     </row>
     <row r="107">
       <c r="A107" s="5" t="str">
-        <v>EQPTZ2501075</v>
+        <v>EFAZZ0001624</v>
       </c>
       <c r="B107" s="5" t="str">
-        <v>800G DR8</v>
+        <v>800G 2XFR4</v>
       </c>
       <c r="C107" s="6" t="str">
-        <v>#02</v>
+        <v>#13</v>
       </c>
       <c r="D107" s="5" t="str">
         <v>TX AA</v>
@@ -2023,13 +2023,13 @@
     </row>
     <row r="108">
       <c r="A108" s="5" t="str">
-        <v>EQPTZ2501076</v>
+        <v>EQPTZ2500008</v>
       </c>
       <c r="B108" s="5" t="str">
-        <v>800G DR8</v>
+        <v>800G 2XFR4</v>
       </c>
       <c r="C108" s="6" t="str">
-        <v>#03</v>
+        <v>#14</v>
       </c>
       <c r="D108" s="5" t="str">
         <v>TX AA</v>
@@ -2037,13 +2037,13 @@
     </row>
     <row r="109">
       <c r="A109" s="5" t="str">
-        <v>EQPTZ2501080</v>
+        <v>EQPTZ2501067</v>
       </c>
       <c r="B109" s="5" t="str">
-        <v>800G DR8</v>
+        <v>800G 2XFR4</v>
       </c>
       <c r="C109" s="6" t="str">
-        <v>#04</v>
+        <v>#15</v>
       </c>
       <c r="D109" s="5" t="str">
         <v>TX AA</v>
@@ -2051,13 +2051,13 @@
     </row>
     <row r="110">
       <c r="A110" s="5" t="str">
-        <v>EQPTZ2501068</v>
+        <v>EQPTZ2501088</v>
       </c>
       <c r="B110" s="5" t="str">
-        <v>800G DR8</v>
+        <v>800G 2XFR4</v>
       </c>
       <c r="C110" s="6" t="str">
-        <v>#05</v>
+        <v>#16</v>
       </c>
       <c r="D110" s="5" t="str">
         <v>TX AA</v>
@@ -2065,13 +2065,13 @@
     </row>
     <row r="111">
       <c r="A111" s="5" t="str">
-        <v>EQPTZ2501088</v>
+        <v>EFAZZ0000868</v>
       </c>
       <c r="B111" s="5" t="str">
-        <v>800G DR8</v>
+        <v>800G 2XFR4</v>
       </c>
       <c r="C111" s="6" t="str">
-        <v>#06</v>
+        <v>#17</v>
       </c>
       <c r="D111" s="5" t="str">
         <v>TX AA</v>
@@ -2079,13 +2079,13 @@
     </row>
     <row r="112">
       <c r="A112" s="5" t="str">
-        <v>EQPTZ2501086</v>
+        <v>EQPTZ2501080</v>
       </c>
       <c r="B112" s="5" t="str">
-        <v>800G DR8</v>
+        <v>800G 2XFR4</v>
       </c>
       <c r="C112" s="6" t="str">
-        <v>#07</v>
+        <v>#18</v>
       </c>
       <c r="D112" s="5" t="str">
         <v>TX AA</v>
@@ -2093,181 +2093,181 @@
     </row>
     <row r="113">
       <c r="A113" s="5" t="str">
-        <v>EQPTZ2501085</v>
+        <v/>
       </c>
       <c r="B113" s="5" t="str">
-        <v>800G DR8</v>
+        <v/>
       </c>
       <c r="C113" s="6" t="str">
-        <v>#08</v>
+        <v/>
       </c>
       <c r="D113" s="5" t="str">
-        <v>TX AA</v>
+        <v/>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="5" t="str">
-        <v>EQPTZ2501084</v>
+        <v>EQPTZ2400148</v>
       </c>
       <c r="B114" s="5" t="str">
-        <v>800G DR8</v>
+        <v>800G 2XFR4</v>
       </c>
       <c r="C114" s="6" t="str">
-        <v>#09</v>
+        <v>#01</v>
       </c>
       <c r="D114" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="5" t="str">
-        <v>EQPTZ2501073</v>
+        <v>EFAZZ0001769</v>
       </c>
       <c r="B115" s="5" t="str">
-        <v>800G DR8</v>
+        <v>800G 2XFR4</v>
       </c>
       <c r="C115" s="6" t="str">
-        <v>#10</v>
+        <v>#02</v>
       </c>
       <c r="D115" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="5" t="str">
-        <v>EQPTZ2501087</v>
+        <v>EZDYH2400071</v>
       </c>
       <c r="B116" s="5" t="str">
-        <v>800G DR8</v>
+        <v>800G 2XFR4</v>
       </c>
       <c r="C116" s="6" t="str">
-        <v>#11</v>
+        <v>#03</v>
       </c>
       <c r="D116" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="5" t="str">
-        <v>EQPTZ2501091</v>
+        <v>EZDYH2400085</v>
       </c>
       <c r="B117" s="5" t="str">
-        <v>800G DR8</v>
+        <v>800G 2XFR4</v>
       </c>
       <c r="C117" s="6" t="str">
-        <v>#12</v>
+        <v>#04</v>
       </c>
       <c r="D117" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="5" t="str">
-        <v>EQPTZ2501090</v>
+        <v>EZDYH2400090</v>
       </c>
       <c r="B118" s="5" t="str">
-        <v>800G DR8</v>
+        <v>800G 2XFR4</v>
       </c>
       <c r="C118" s="6" t="str">
-        <v>#13</v>
+        <v>#05</v>
       </c>
       <c r="D118" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="5" t="str">
-        <v>EQPTZ2501098</v>
+        <v>EZDYH2400080</v>
       </c>
       <c r="B119" s="5" t="str">
-        <v>800G DR8</v>
+        <v>800G 2XFR4</v>
       </c>
       <c r="C119" s="6" t="str">
-        <v>#15</v>
+        <v>#06</v>
       </c>
       <c r="D119" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="5" t="str">
-        <v>EZDYH2400213</v>
+        <v>EZDYH2400054</v>
       </c>
       <c r="B120" s="5" t="str">
-        <v>800G DR8</v>
+        <v>800G 2XFR4</v>
       </c>
       <c r="C120" s="6" t="str">
-        <v>#18</v>
+        <v>#07</v>
       </c>
       <c r="D120" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="5" t="str">
-        <v>EQPTZ2501101</v>
+        <v>EZDYH2400096</v>
       </c>
       <c r="B121" s="5" t="str">
-        <v>800G DR8</v>
+        <v>800G 2XFR4</v>
       </c>
       <c r="C121" s="6" t="str">
-        <v>#19</v>
+        <v>#08</v>
       </c>
       <c r="D121" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="5" t="str">
-        <v>EFAZZ0001607</v>
+        <v>EQPTZ2501104</v>
       </c>
       <c r="B122" s="5" t="str">
-        <v>800G DR8</v>
+        <v>800G 2XFR4</v>
       </c>
       <c r="C122" s="6" t="str">
-        <v>#22</v>
+        <v>#09</v>
       </c>
       <c r="D122" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="5" t="str">
-        <v>EFAZZ0001608</v>
+        <v>EQPTZ2501102</v>
       </c>
       <c r="B123" s="5" t="str">
-        <v>800G DR8</v>
+        <v>800G 2XFR4</v>
       </c>
       <c r="C123" s="6" t="str">
-        <v>#24</v>
+        <v>#10</v>
       </c>
       <c r="D123" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="5" t="str">
-        <v>EYHJE2400044</v>
+        <v/>
       </c>
       <c r="B124" s="5" t="str">
-        <v>800G DR8</v>
+        <v/>
       </c>
       <c r="C124" s="6" t="str">
-        <v>#25</v>
+        <v/>
       </c>
       <c r="D124" s="5" t="str">
-        <v>TX AA</v>
+        <v/>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="5" t="str">
-        <v>EFAZZ0001606</v>
+        <v>EFAZZ0000816</v>
       </c>
       <c r="B125" s="5" t="str">
-        <v>800G DR8</v>
+        <v>400G FR4</v>
       </c>
       <c r="C125" s="6" t="str">
-        <v>#26</v>
+        <v>#01</v>
       </c>
       <c r="D125" s="5" t="str">
         <v>TX AA</v>
@@ -2275,13 +2275,13 @@
     </row>
     <row r="126">
       <c r="A126" s="5" t="str">
-        <v>EYHJE2400018</v>
+        <v>EFAZZ0001032</v>
       </c>
       <c r="B126" s="5" t="str">
-        <v>800G DR8</v>
+        <v>400G FR4</v>
       </c>
       <c r="C126" s="6" t="str">
-        <v>#27</v>
+        <v>#02</v>
       </c>
       <c r="D126" s="5" t="str">
         <v>TX AA</v>
@@ -2289,44 +2289,44 @@
     </row>
     <row r="127">
       <c r="A127" s="5" t="str">
-        <v>EFAZZ0000854</v>
+        <v/>
       </c>
       <c r="B127" s="5" t="str">
-        <v>800G DR8</v>
+        <v/>
       </c>
       <c r="C127" s="6" t="str">
-        <v>#30</v>
+        <v/>
       </c>
       <c r="D127" s="5" t="str">
-        <v>TX AA</v>
+        <v/>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="5" t="str">
-        <v>EFAZZ0000852</v>
+        <v>EFAZZ0001559</v>
       </c>
       <c r="B128" s="5" t="str">
-        <v>800G DR8</v>
+        <v>200G AOC GEN2</v>
       </c>
       <c r="C128" s="6" t="str">
-        <v>#31</v>
+        <v>#00</v>
       </c>
       <c r="D128" s="5" t="str">
-        <v>TX AA</v>
+        <v>MM AA</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="5" t="str">
-        <v>EFAZZ0001734</v>
+        <v>EZDYH0000111</v>
       </c>
       <c r="B129" s="5" t="str">
-        <v>800G DR8</v>
+        <v>200G AOC GEN2</v>
       </c>
       <c r="C129" s="6" t="str">
-        <v>#32</v>
+        <v>#00</v>
       </c>
       <c r="D129" s="5" t="str">
-        <v>TX AA</v>
+        <v>MM AA</v>
       </c>
     </row>
     <row r="130">
@@ -2345,13 +2345,13 @@
     </row>
     <row r="131">
       <c r="A131" s="5" t="str">
-        <v>EFAZZ2400673</v>
+        <v>EFAZZ0000820</v>
       </c>
       <c r="B131" s="5" t="str">
-        <v>800G 2XFR4</v>
+        <v>400G CGR4+</v>
       </c>
       <c r="C131" s="6" t="str">
-        <v>#01</v>
+        <v>#05</v>
       </c>
       <c r="D131" s="5" t="str">
         <v>TX AA</v>
@@ -2359,13 +2359,13 @@
     </row>
     <row r="132">
       <c r="A132" s="5" t="str">
-        <v>EQPTZ2500004</v>
+        <v>EFAZZ0000851</v>
       </c>
       <c r="B132" s="5" t="str">
-        <v>800G 2XFR4</v>
+        <v>400G CGR4+</v>
       </c>
       <c r="C132" s="6" t="str">
-        <v>#02</v>
+        <v>#06</v>
       </c>
       <c r="D132" s="5" t="str">
         <v>TX AA</v>
@@ -2373,13 +2373,13 @@
     </row>
     <row r="133">
       <c r="A133" s="5" t="str">
-        <v>EQPTZ2500005</v>
+        <v>EZDYH0000057</v>
       </c>
       <c r="B133" s="5" t="str">
-        <v>800G 2XFR4</v>
+        <v>400G CGR4+</v>
       </c>
       <c r="C133" s="6" t="str">
-        <v>#03</v>
+        <v>#08</v>
       </c>
       <c r="D133" s="5" t="str">
         <v>TX AA</v>
@@ -2387,13 +2387,13 @@
     </row>
     <row r="134">
       <c r="A134" s="5" t="str">
-        <v>EZDYH2400051</v>
+        <v>EZDYH0000066</v>
       </c>
       <c r="B134" s="5" t="str">
-        <v>800G 2XFR4</v>
+        <v>400G CGR4+</v>
       </c>
       <c r="C134" s="6" t="str">
-        <v>#04</v>
+        <v>#09</v>
       </c>
       <c r="D134" s="5" t="str">
         <v>TX AA</v>
@@ -2401,181 +2401,181 @@
     </row>
     <row r="135">
       <c r="A135" s="5" t="str">
-        <v>EQPTZ2400292</v>
+        <v/>
       </c>
       <c r="B135" s="5" t="str">
-        <v>800G 2XFR4</v>
+        <v/>
       </c>
       <c r="C135" s="6" t="str">
-        <v>#05</v>
+        <v/>
       </c>
       <c r="D135" s="5" t="str">
-        <v>TX AA</v>
+        <v/>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="5" t="str">
-        <v>EZDYH2400088</v>
+        <v>EFAZZ0001006</v>
       </c>
       <c r="B136" s="5" t="str">
-        <v>800G 2XFR4</v>
+        <v>400G DR4</v>
       </c>
       <c r="C136" s="6" t="str">
-        <v>#06</v>
+        <v>#15</v>
       </c>
       <c r="D136" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="5" t="str">
-        <v>EZDYH2400191</v>
+        <v>EFAZZ0001005</v>
       </c>
       <c r="B137" s="5" t="str">
-        <v>800G 2XFR4</v>
+        <v>400G DR4</v>
       </c>
       <c r="C137" s="6" t="str">
-        <v>#07</v>
+        <v>#16</v>
       </c>
       <c r="D137" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="5" t="str">
-        <v>EQPTZ2501089</v>
+        <v>EFAZZ0000282</v>
       </c>
       <c r="B138" s="5" t="str">
-        <v>800G 2XFR4</v>
+        <v>400G DR4</v>
       </c>
       <c r="C138" s="6" t="str">
-        <v>#08</v>
+        <v>#18</v>
       </c>
       <c r="D138" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="5" t="str">
-        <v>EQPTZ2501093</v>
+        <v>EFAZZ0000924</v>
       </c>
       <c r="B139" s="5" t="str">
-        <v>800G 2XFR4</v>
+        <v>400G DR4</v>
       </c>
       <c r="C139" s="6" t="str">
-        <v>#09</v>
+        <v>#19</v>
       </c>
       <c r="D139" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="5" t="str">
-        <v>EQPTZ2500009</v>
+        <v>EFAZZ0001042</v>
       </c>
       <c r="B140" s="5" t="str">
-        <v>800G 2XFR4</v>
+        <v>400G DR4</v>
       </c>
       <c r="C140" s="6" t="str">
-        <v>#10</v>
+        <v>#26</v>
       </c>
       <c r="D140" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="5" t="str">
-        <v>EQPTZ2501077</v>
+        <v>EFAZZ0001043</v>
       </c>
       <c r="B141" s="5" t="str">
-        <v>800G 2XFR4</v>
+        <v>400G DR4</v>
       </c>
       <c r="C141" s="6" t="str">
-        <v>#11</v>
+        <v>#27</v>
       </c>
       <c r="D141" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="5" t="str">
-        <v>EQPTZ2501079</v>
+        <v>EFAZZ0001045</v>
       </c>
       <c r="B142" s="5" t="str">
-        <v>800G 2XFR4</v>
+        <v>400G DR4</v>
       </c>
       <c r="C142" s="6" t="str">
-        <v>#12</v>
+        <v>#28</v>
       </c>
       <c r="D142" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="5" t="str">
-        <v>EFAZZ0001624</v>
+        <v>EFAZZ0001044</v>
       </c>
       <c r="B143" s="5" t="str">
-        <v>800G 2XFR4</v>
+        <v>400G DR4</v>
       </c>
       <c r="C143" s="6" t="str">
-        <v>#13</v>
+        <v>#29</v>
       </c>
       <c r="D143" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="5" t="str">
-        <v>EQPTZ2500008</v>
+        <v>EFAZZ0000922</v>
       </c>
       <c r="B144" s="5" t="str">
-        <v>800G 2XFR4</v>
+        <v>400G DR4</v>
       </c>
       <c r="C144" s="6" t="str">
-        <v>#14</v>
+        <v>#37</v>
       </c>
       <c r="D144" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="5" t="str">
-        <v>EQPTZ2501067</v>
+        <v>EFAZZ0001849</v>
       </c>
       <c r="B145" s="5" t="str">
-        <v>800G 2XFR4</v>
+        <v>400G DR4</v>
       </c>
       <c r="C145" s="6" t="str">
-        <v>#15</v>
+        <v>#48</v>
       </c>
       <c r="D145" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="5" t="str">
-        <v/>
+        <v>EFAZZ0001856</v>
       </c>
       <c r="B146" s="5" t="str">
-        <v/>
+        <v>400G DR4</v>
       </c>
       <c r="C146" s="6" t="str">
-        <v/>
+        <v>#49</v>
       </c>
       <c r="D146" s="5" t="str">
-        <v/>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="5" t="str">
-        <v>EQPTZ2400148</v>
+        <v>EFAZZ0001855</v>
       </c>
       <c r="B147" s="5" t="str">
-        <v>800G 2XFR4</v>
+        <v>400G DR4</v>
       </c>
       <c r="C147" s="6" t="str">
-        <v>#01</v>
+        <v>#51</v>
       </c>
       <c r="D147" s="5" t="str">
         <v>TRX FA</v>
@@ -2583,13 +2583,13 @@
     </row>
     <row r="148">
       <c r="A148" s="5" t="str">
-        <v>EFAZZ0001769</v>
+        <v>EFAZZ0001848</v>
       </c>
       <c r="B148" s="5" t="str">
-        <v>800G 2XFR4</v>
+        <v>400G DR4</v>
       </c>
       <c r="C148" s="6" t="str">
-        <v>#02</v>
+        <v>#52</v>
       </c>
       <c r="D148" s="5" t="str">
         <v>TRX FA</v>
@@ -2597,13 +2597,13 @@
     </row>
     <row r="149">
       <c r="A149" s="5" t="str">
-        <v>EZDYH2400071</v>
+        <v>EFAZZ0001847</v>
       </c>
       <c r="B149" s="5" t="str">
-        <v>800G 2XFR4</v>
+        <v>400G DR4</v>
       </c>
       <c r="C149" s="6" t="str">
-        <v>#03</v>
+        <v>#53</v>
       </c>
       <c r="D149" s="5" t="str">
         <v>TRX FA</v>
@@ -2611,13 +2611,13 @@
     </row>
     <row r="150">
       <c r="A150" s="5" t="str">
-        <v>EZDYH2400085</v>
+        <v>EFAZZ0001846</v>
       </c>
       <c r="B150" s="5" t="str">
-        <v>800G 2XFR4</v>
+        <v>400G DR4</v>
       </c>
       <c r="C150" s="6" t="str">
-        <v>#04</v>
+        <v>#54</v>
       </c>
       <c r="D150" s="5" t="str">
         <v>TRX FA</v>
@@ -2625,83 +2625,83 @@
     </row>
     <row r="151">
       <c r="A151" s="5" t="str">
-        <v>EZDYH2400090</v>
+        <v/>
       </c>
       <c r="B151" s="5" t="str">
-        <v>800G 2XFR4</v>
+        <v/>
       </c>
       <c r="C151" s="6" t="str">
-        <v>#05</v>
+        <v/>
       </c>
       <c r="D151" s="5" t="str">
-        <v>TRX FA</v>
+        <v/>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="5" t="str">
-        <v>EZDYH2400080</v>
+        <v>EFAZZ0001646</v>
       </c>
       <c r="B152" s="5" t="str">
-        <v>800G 2XFR4</v>
+        <v>400G DR4</v>
       </c>
       <c r="C152" s="6" t="str">
-        <v>#06</v>
+        <v>#35</v>
       </c>
       <c r="D152" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="5" t="str">
-        <v>EZDYH2400054</v>
+        <v>EFAZZ0001565</v>
       </c>
       <c r="B153" s="5" t="str">
-        <v>800G 2XFR4</v>
+        <v>400G DR4</v>
       </c>
       <c r="C153" s="6" t="str">
-        <v>#07</v>
+        <v>#36</v>
       </c>
       <c r="D153" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="5" t="str">
-        <v>EZDYH2400096</v>
+        <v>EFAZZ0001600</v>
       </c>
       <c r="B154" s="5" t="str">
-        <v>800G 2XFR4</v>
+        <v>400G DR4</v>
       </c>
       <c r="C154" s="6" t="str">
-        <v>#08</v>
+        <v>#37</v>
       </c>
       <c r="D154" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="5" t="str">
-        <v>EQPTZ2501104</v>
+        <v/>
       </c>
       <c r="B155" s="5" t="str">
-        <v>800G 2XFR4</v>
+        <v/>
       </c>
       <c r="C155" s="6" t="str">
-        <v>#09</v>
+        <v/>
       </c>
       <c r="D155" s="5" t="str">
-        <v>TRX FA</v>
+        <v/>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="5" t="str">
-        <v>EQPTZ2501102</v>
+        <v>EFAZZ0001845</v>
       </c>
       <c r="B156" s="5" t="str">
-        <v>800G 2XFR4</v>
+        <v>100G DR1</v>
       </c>
       <c r="C156" s="6" t="str">
-        <v>#10</v>
+        <v>#01</v>
       </c>
       <c r="D156" s="5" t="str">
         <v>TRX FA</v>
@@ -2709,44 +2709,44 @@
     </row>
     <row r="157">
       <c r="A157" s="5" t="str">
-        <v/>
+        <v>EFAZZ0000842</v>
       </c>
       <c r="B157" s="5" t="str">
-        <v/>
+        <v>100G DR1</v>
       </c>
       <c r="C157" s="6" t="str">
-        <v/>
+        <v>#02</v>
       </c>
       <c r="D157" s="5" t="str">
-        <v/>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="5" t="str">
-        <v>EFAZZ2400191</v>
+        <v/>
       </c>
       <c r="B158" s="5" t="str">
-        <v>800G DR8 AWS</v>
+        <v/>
       </c>
       <c r="C158" s="6" t="str">
-        <v>#01</v>
+        <v/>
       </c>
       <c r="D158" s="5" t="str">
-        <v>TRX FA</v>
+        <v/>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="5" t="str">
-        <v>EZDYH2400192</v>
+        <v>EYHJE2400025</v>
       </c>
       <c r="B159" s="5" t="str">
-        <v>800G DR8 AWS</v>
+        <v>800G 2XFR4 GEN1</v>
       </c>
       <c r="C159" s="6" t="str">
-        <v>#02</v>
+        <v>#01</v>
       </c>
       <c r="D159" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA  [ NPI ]</v>
       </c>
     </row>
     <row r="160">
@@ -2765,195 +2765,195 @@
     </row>
     <row r="161">
       <c r="A161" s="5" t="str">
-        <v>EQPTZ2501083</v>
+        <v>EFAZZ0001772</v>
       </c>
       <c r="B161" s="5" t="str">
-        <v>800G DR8 AWS</v>
+        <v>800G 2XFR4 GEN1</v>
       </c>
       <c r="C161" s="6" t="str">
         <v>#02</v>
       </c>
       <c r="D161" s="5" t="str">
-        <v>TX AA</v>
+        <v>TX AA [ NPI ]</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="5" t="str">
-        <v/>
+        <v>EFAZZ0001753</v>
       </c>
       <c r="B162" s="5" t="str">
-        <v/>
+        <v>800G 2XFR4 GEN1</v>
       </c>
       <c r="C162" s="6" t="str">
-        <v/>
+        <v>#04</v>
       </c>
       <c r="D162" s="5" t="str">
-        <v/>
+        <v>TX AA [ NPI ]</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="5" t="str">
-        <v>EZDYH2400053</v>
+        <v/>
       </c>
       <c r="B163" s="5" t="str">
-        <v>400G FR4 FA</v>
+        <v/>
       </c>
       <c r="C163" s="6" t="str">
-        <v>#01</v>
+        <v/>
       </c>
       <c r="D163" s="5" t="str">
-        <v>TRX FA</v>
+        <v/>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="5" t="str">
-        <v/>
+        <v>EFAZZ0001689</v>
       </c>
       <c r="B164" s="5" t="str">
-        <v/>
+        <v>800G 2XFR4 GEN1</v>
       </c>
       <c r="C164" s="6" t="str">
-        <v/>
+        <v>#03</v>
       </c>
       <c r="D164" s="5" t="str">
-        <v/>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="5" t="str">
-        <v>EFAZZ0001032</v>
+        <v/>
       </c>
       <c r="B165" s="5" t="str">
-        <v>400G FR4</v>
+        <v/>
       </c>
       <c r="C165" s="6" t="str">
-        <v>#02</v>
+        <v/>
       </c>
       <c r="D165" s="5" t="str">
-        <v>TX AA</v>
+        <v/>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="5" t="str">
-        <v/>
+        <v>EQPTZ2400147</v>
       </c>
       <c r="B166" s="5" t="str">
-        <v/>
+        <v>8X200G 2XDR4</v>
       </c>
       <c r="C166" s="6" t="str">
-        <v/>
+        <v>#01</v>
       </c>
       <c r="D166" s="5" t="str">
-        <v/>
+        <v>TRX FA [ NPI ]</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="5" t="str">
-        <v>EZDYH2400056</v>
+        <v/>
       </c>
       <c r="B167" s="5" t="str">
-        <v>400G FR4 OUT</v>
+        <v/>
       </c>
       <c r="C167" s="6" t="str">
-        <v>#02</v>
+        <v/>
       </c>
       <c r="D167" s="5" t="str">
-        <v>OUT LEN</v>
+        <v/>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="5" t="str">
-        <v/>
+        <v>EZDYH2400214</v>
       </c>
       <c r="B168" s="5" t="str">
-        <v/>
+        <v>8X200G 2XDR4</v>
       </c>
       <c r="C168" s="6" t="str">
-        <v/>
+        <v>#01</v>
       </c>
       <c r="D168" s="5" t="str">
-        <v/>
+        <v>MPD [ NPI ]</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="5" t="str">
-        <v>EFAZZ0001703</v>
+        <v/>
       </c>
       <c r="B169" s="5" t="str">
-        <v>400G Q112 DR4</v>
+        <v/>
       </c>
       <c r="C169" s="6" t="str">
-        <v>#00</v>
+        <v/>
       </c>
       <c r="D169" s="5" t="str">
-        <v>TRX FA [ NPI ]</v>
+        <v/>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="5" t="str">
-        <v/>
+        <v>EQPTZ2501078</v>
       </c>
       <c r="B170" s="5" t="str">
-        <v/>
+        <v>8X200G DR8 TRO</v>
       </c>
       <c r="C170" s="6" t="str">
-        <v/>
+        <v>#01</v>
       </c>
       <c r="D170" s="5" t="str">
-        <v/>
+        <v>TRX FA [ NPI ]</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="5" t="str">
-        <v>EZDYH2400196</v>
+        <v/>
       </c>
       <c r="B171" s="5" t="str">
-        <v>800G 2XFR4 OUT</v>
+        <v/>
       </c>
       <c r="C171" s="6" t="str">
-        <v>#01</v>
+        <v/>
       </c>
       <c r="D171" s="5" t="str">
-        <v>OUT LEN</v>
+        <v/>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="5" t="str">
-        <v>EQPTZ2500003</v>
+        <v>EQPTZ2501084</v>
       </c>
       <c r="B172" s="5" t="str">
-        <v>800G 2XFR4 OUT</v>
+        <v>8X200G DR8 TRO</v>
       </c>
       <c r="C172" s="6" t="str">
-        <v>#02</v>
+        <v>#01</v>
       </c>
       <c r="D172" s="5" t="str">
-        <v>OUT LEN</v>
+        <v>MPD [ NPI ]</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="5" t="str">
-        <v>EZDYH2400194</v>
+        <v/>
       </c>
       <c r="B173" s="5" t="str">
-        <v>800G 2XFR4 OUT</v>
+        <v/>
       </c>
       <c r="C173" s="6" t="str">
-        <v>#03</v>
+        <v/>
       </c>
       <c r="D173" s="5" t="str">
-        <v>OUT LEN</v>
+        <v/>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="5" t="str">
-        <v>EQPTZ2400232</v>
+        <v>EZDYH2400196</v>
       </c>
       <c r="B174" s="5" t="str">
         <v>800G 2XFR4 OUT</v>
       </c>
       <c r="C174" s="6" t="str">
-        <v>#04</v>
+        <v>#01</v>
       </c>
       <c r="D174" s="5" t="str">
         <v>OUT LEN</v>
@@ -2961,13 +2961,13 @@
     </row>
     <row r="175">
       <c r="A175" s="5" t="str">
-        <v>EZDYH2400195</v>
+        <v>EQPTZ2500003</v>
       </c>
       <c r="B175" s="5" t="str">
         <v>800G 2XFR4 OUT</v>
       </c>
       <c r="C175" s="6" t="str">
-        <v>#05</v>
+        <v>#02</v>
       </c>
       <c r="D175" s="5" t="str">
         <v>OUT LEN</v>
@@ -2975,13 +2975,13 @@
     </row>
     <row r="176">
       <c r="A176" s="5" t="str">
-        <v>EQPTZ2501071</v>
+        <v>EZDYH2400194</v>
       </c>
       <c r="B176" s="5" t="str">
         <v>800G 2XFR4 OUT</v>
       </c>
       <c r="C176" s="6" t="str">
-        <v>#06</v>
+        <v>#03</v>
       </c>
       <c r="D176" s="5" t="str">
         <v>OUT LEN</v>
@@ -2989,13 +2989,13 @@
     </row>
     <row r="177">
       <c r="A177" s="5" t="str">
-        <v>EQPTZ2501070</v>
+        <v>EQPTZ2400232</v>
       </c>
       <c r="B177" s="5" t="str">
         <v>800G 2XFR4 OUT</v>
       </c>
       <c r="C177" s="6" t="str">
-        <v>#07</v>
+        <v>#04</v>
       </c>
       <c r="D177" s="5" t="str">
         <v>OUT LEN</v>
@@ -3003,181 +3003,181 @@
     </row>
     <row r="178">
       <c r="A178" s="5" t="str">
-        <v/>
+        <v>EZDYH2400195</v>
       </c>
       <c r="B178" s="5" t="str">
-        <v/>
+        <v>800G 2XFR4 OUT</v>
       </c>
       <c r="C178" s="6" t="str">
-        <v/>
+        <v>#05</v>
       </c>
       <c r="D178" s="5" t="str">
-        <v/>
+        <v>OUT LEN</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="5" t="str">
-        <v>EFAZZ0001753</v>
+        <v>EQPTZ2501071</v>
       </c>
       <c r="B179" s="5" t="str">
-        <v>800G CDGR4+</v>
+        <v>800G 2XFR4 OUT</v>
       </c>
       <c r="C179" s="6" t="str">
-        <v>#01</v>
+        <v>#06</v>
       </c>
       <c r="D179" s="5" t="str">
-        <v>TX AA</v>
+        <v>OUT LEN</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="5" t="str">
-        <v>EFAZZ0001764</v>
+        <v>EQPTZ2501070</v>
       </c>
       <c r="B180" s="5" t="str">
-        <v>800G CDGR4+</v>
+        <v>800G 2XFR4 OUT</v>
       </c>
       <c r="C180" s="6" t="str">
-        <v>#02</v>
+        <v>#07</v>
       </c>
       <c r="D180" s="5" t="str">
-        <v>TX AA</v>
+        <v>OUT LEN</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="5" t="str">
-        <v>EFAZZ0001758</v>
+        <v>EQPTZ2501073</v>
       </c>
       <c r="B181" s="5" t="str">
-        <v>800G CDGR4+</v>
+        <v>800G 2XFR4 OUT</v>
       </c>
       <c r="C181" s="6" t="str">
-        <v>#03</v>
+        <v>#08</v>
       </c>
       <c r="D181" s="5" t="str">
-        <v>TX AA</v>
+        <v>OUT LEN</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="5" t="str">
-        <v>EFAZZ0000302</v>
+        <v>EQPTZ2501068</v>
       </c>
       <c r="B182" s="5" t="str">
-        <v>800G CDGR4+</v>
+        <v>800G 2XFR4 OUT</v>
       </c>
       <c r="C182" s="6" t="str">
-        <v>#04</v>
+        <v>#09</v>
       </c>
       <c r="D182" s="5" t="str">
-        <v>TX AA</v>
+        <v>OUT LEN</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="5" t="str">
-        <v>EFAZZ0000301</v>
+        <v/>
       </c>
       <c r="B183" s="5" t="str">
-        <v>800G CDGR4+</v>
+        <v/>
       </c>
       <c r="C183" s="6" t="str">
-        <v>#05</v>
+        <v/>
       </c>
       <c r="D183" s="5" t="str">
-        <v>TX AA</v>
+        <v/>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="5" t="str">
-        <v>EFAZZ0000555</v>
+        <v>EZDYH2400053</v>
       </c>
       <c r="B184" s="5" t="str">
-        <v>800G CDGR4+</v>
+        <v>400G FR4 FA</v>
       </c>
       <c r="C184" s="6" t="str">
-        <v>#06</v>
+        <v>#01</v>
       </c>
       <c r="D184" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="5" t="str">
-        <v>EFAZZ0000807</v>
+        <v/>
       </c>
       <c r="B185" s="5" t="str">
-        <v>800G CDGR4+</v>
+        <v/>
       </c>
       <c r="C185" s="6" t="str">
-        <v>#07</v>
+        <v/>
       </c>
       <c r="D185" s="5" t="str">
-        <v>TX AA</v>
+        <v/>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="5" t="str">
-        <v>EFAZZ0000588</v>
+        <v>EZDYH2400056</v>
       </c>
       <c r="B186" s="5" t="str">
-        <v>800G CDGR4+</v>
+        <v>400G FR4 OUT</v>
       </c>
       <c r="C186" s="6" t="str">
-        <v>#08</v>
+        <v>#02</v>
       </c>
       <c r="D186" s="5" t="str">
-        <v>TX AA</v>
+        <v>OUT LEN</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="5" t="str">
-        <v>EFAZZ0000809</v>
+        <v/>
       </c>
       <c r="B187" s="5" t="str">
-        <v>800G CDGR4+</v>
+        <v/>
       </c>
       <c r="C187" s="6" t="str">
-        <v>#09</v>
+        <v/>
       </c>
       <c r="D187" s="5" t="str">
-        <v>TX AA</v>
+        <v/>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="5" t="str">
-        <v>EFAZZ0001762</v>
+        <v>EFAZZ0001703</v>
       </c>
       <c r="B188" s="5" t="str">
-        <v>800G CDGR4+</v>
+        <v>400G Q112 DR4</v>
       </c>
       <c r="C188" s="6" t="str">
-        <v>#10</v>
+        <v>#00</v>
       </c>
       <c r="D188" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA [ NPI ]</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="5" t="str">
-        <v>EFAZZ0000554</v>
+        <v/>
       </c>
       <c r="B189" s="5" t="str">
-        <v>800G CDGR4+</v>
+        <v/>
       </c>
       <c r="C189" s="6" t="str">
-        <v>#11</v>
+        <v/>
       </c>
       <c r="D189" s="5" t="str">
-        <v>TX AA</v>
+        <v/>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="5" t="str">
-        <v>EFAZZ0001689</v>
+        <v>EFAZZ0001764</v>
       </c>
       <c r="B190" s="5" t="str">
         <v>800G CDGR4+</v>
       </c>
       <c r="C190" s="6" t="str">
-        <v>#12</v>
+        <v>#02</v>
       </c>
       <c r="D190" s="5" t="str">
         <v>TX AA</v>
@@ -3185,13 +3185,13 @@
     </row>
     <row r="191">
       <c r="A191" s="5" t="str">
-        <v>EFAZZ0001680</v>
+        <v>EFAZZ0001758</v>
       </c>
       <c r="B191" s="5" t="str">
         <v>800G CDGR4+</v>
       </c>
       <c r="C191" s="6" t="str">
-        <v>#13</v>
+        <v>#03</v>
       </c>
       <c r="D191" s="5" t="str">
         <v>TX AA</v>
@@ -3199,13 +3199,13 @@
     </row>
     <row r="192">
       <c r="A192" s="5" t="str">
-        <v>EFAZZ0001690</v>
+        <v>EFAZZ0000302</v>
       </c>
       <c r="B192" s="5" t="str">
         <v>800G CDGR4+</v>
       </c>
       <c r="C192" s="6" t="str">
-        <v>#14</v>
+        <v>#04</v>
       </c>
       <c r="D192" s="5" t="str">
         <v>TX AA</v>
@@ -3213,13 +3213,13 @@
     </row>
     <row r="193">
       <c r="A193" s="5" t="str">
-        <v>EFAZZ0001712</v>
+        <v>EFAZZ0000301</v>
       </c>
       <c r="B193" s="5" t="str">
         <v>800G CDGR4+</v>
       </c>
       <c r="C193" s="6" t="str">
-        <v>#15</v>
+        <v>#05</v>
       </c>
       <c r="D193" s="5" t="str">
         <v>TX AA</v>
@@ -3227,13 +3227,13 @@
     </row>
     <row r="194">
       <c r="A194" s="5" t="str">
-        <v>EFAZZ0001763</v>
+        <v>EFAZZ0000555</v>
       </c>
       <c r="B194" s="5" t="str">
         <v>800G CDGR4+</v>
       </c>
       <c r="C194" s="6" t="str">
-        <v>#16</v>
+        <v>#06</v>
       </c>
       <c r="D194" s="5" t="str">
         <v>TX AA</v>
@@ -3241,13 +3241,13 @@
     </row>
     <row r="195">
       <c r="A195" s="5" t="str">
-        <v>EFAZZ0001761</v>
+        <v>EFAZZ0000807</v>
       </c>
       <c r="B195" s="5" t="str">
         <v>800G CDGR4+</v>
       </c>
       <c r="C195" s="6" t="str">
-        <v>#17</v>
+        <v>#07</v>
       </c>
       <c r="D195" s="5" t="str">
         <v>TX AA</v>
@@ -3255,13 +3255,13 @@
     </row>
     <row r="196">
       <c r="A196" s="5" t="str">
-        <v>EFAZZ0001788</v>
+        <v>EFAZZ0000588</v>
       </c>
       <c r="B196" s="5" t="str">
         <v>800G CDGR4+</v>
       </c>
       <c r="C196" s="6" t="str">
-        <v>#18</v>
+        <v>#08</v>
       </c>
       <c r="D196" s="5" t="str">
         <v>TX AA</v>
@@ -3269,13 +3269,13 @@
     </row>
     <row r="197">
       <c r="A197" s="5" t="str">
-        <v>EFAZZ0001773</v>
+        <v>EFAZZ0000809</v>
       </c>
       <c r="B197" s="5" t="str">
         <v>800G CDGR4+</v>
       </c>
       <c r="C197" s="6" t="str">
-        <v>#19</v>
+        <v>#09</v>
       </c>
       <c r="D197" s="5" t="str">
         <v>TX AA</v>
@@ -3283,13 +3283,13 @@
     </row>
     <row r="198">
       <c r="A198" s="5" t="str">
-        <v>EFAZZ0001790</v>
+        <v>EFAZZ0001762</v>
       </c>
       <c r="B198" s="5" t="str">
         <v>800G CDGR4+</v>
       </c>
       <c r="C198" s="6" t="str">
-        <v>#20</v>
+        <v>#10</v>
       </c>
       <c r="D198" s="5" t="str">
         <v>TX AA</v>
@@ -3297,153 +3297,153 @@
     </row>
     <row r="199">
       <c r="A199" s="5" t="str">
-        <v/>
+        <v>EFAZZ0000554</v>
       </c>
       <c r="B199" s="5" t="str">
-        <v/>
+        <v>800G CDGR4+</v>
       </c>
       <c r="C199" s="6" t="str">
-        <v/>
+        <v>#11</v>
       </c>
       <c r="D199" s="5" t="str">
-        <v/>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="5" t="str">
-        <v>EZDYH0000124</v>
+        <v>EFAZZ0001680</v>
       </c>
       <c r="B200" s="5" t="str">
-        <v>800G PSM8</v>
+        <v>800G CDGR4+</v>
       </c>
       <c r="C200" s="6" t="str">
-        <v>#01</v>
+        <v>#13</v>
       </c>
       <c r="D200" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="5" t="str">
-        <v>EFAZZ2400190</v>
+        <v>EFAZZ0001690</v>
       </c>
       <c r="B201" s="5" t="str">
-        <v>800G PSM8</v>
+        <v>800G CDGR4+</v>
       </c>
       <c r="C201" s="6" t="str">
-        <v>#02</v>
+        <v>#14</v>
       </c>
       <c r="D201" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="5" t="str">
-        <v>EFAZZ2400188</v>
+        <v>EFAZZ0001712</v>
       </c>
       <c r="B202" s="5" t="str">
-        <v>800G PSM8</v>
+        <v>800G CDGR4+</v>
       </c>
       <c r="C202" s="6" t="str">
-        <v>#03</v>
+        <v>#15</v>
       </c>
       <c r="D202" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="5" t="str">
-        <v>EFAZZ2400189</v>
+        <v>EFAZZ0001763</v>
       </c>
       <c r="B203" s="5" t="str">
-        <v>800G PSM8</v>
+        <v>800G CDGR4+</v>
       </c>
       <c r="C203" s="6" t="str">
-        <v>#04</v>
+        <v>#16</v>
       </c>
       <c r="D203" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="5" t="str">
-        <v>EZDYH2400070</v>
+        <v>EFAZZ0001761</v>
       </c>
       <c r="B204" s="5" t="str">
-        <v>800G PSM8</v>
+        <v>800G CDGR4+</v>
       </c>
       <c r="C204" s="6" t="str">
-        <v>#05</v>
+        <v>#17</v>
       </c>
       <c r="D204" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="5" t="str">
-        <v>EFAZZ2400187</v>
+        <v>EFAZZ0001788</v>
       </c>
       <c r="B205" s="5" t="str">
-        <v>800G PSM8</v>
+        <v>800G CDGR4+</v>
       </c>
       <c r="C205" s="6" t="str">
-        <v>#06</v>
+        <v>#18</v>
       </c>
       <c r="D205" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="5" t="str">
-        <v>EFAZZ0001861</v>
+        <v>EFAZZ0001773</v>
       </c>
       <c r="B206" s="5" t="str">
-        <v>800G PSM8</v>
+        <v>800G CDGR4+</v>
       </c>
       <c r="C206" s="6" t="str">
-        <v>#07</v>
+        <v>#19</v>
       </c>
       <c r="D206" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="5" t="str">
-        <v>EZDYH0000119</v>
+        <v>EFAZZ0001790</v>
       </c>
       <c r="B207" s="5" t="str">
-        <v>800G PSM8</v>
+        <v>800G CDGR4+</v>
       </c>
       <c r="C207" s="6" t="str">
-        <v>#07</v>
+        <v>#20</v>
       </c>
       <c r="D207" s="5" t="str">
-        <v>TRX FA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="5" t="str">
-        <v>EZDYH0000126</v>
+        <v/>
       </c>
       <c r="B208" s="5" t="str">
-        <v>800G PSM8</v>
+        <v/>
       </c>
       <c r="C208" s="6" t="str">
-        <v>#08</v>
+        <v/>
       </c>
       <c r="D208" s="5" t="str">
-        <v>TRX FA</v>
+        <v/>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="5" t="str">
-        <v>EFAQA0001820</v>
+        <v>EZDYH0000124</v>
       </c>
       <c r="B209" s="5" t="str">
         <v>800G PSM8</v>
       </c>
       <c r="C209" s="6" t="str">
-        <v>#10</v>
+        <v>#01</v>
       </c>
       <c r="D209" s="5" t="str">
         <v>TRX FA</v>
@@ -3451,13 +3451,13 @@
     </row>
     <row r="210">
       <c r="A210" s="5" t="str">
-        <v>EFAZZ0001768</v>
+        <v>EFAZZ2400190</v>
       </c>
       <c r="B210" s="5" t="str">
         <v>800G PSM8</v>
       </c>
       <c r="C210" s="6" t="str">
-        <v>#11</v>
+        <v>#02</v>
       </c>
       <c r="D210" s="5" t="str">
         <v>TRX FA</v>
@@ -3465,13 +3465,13 @@
     </row>
     <row r="211">
       <c r="A211" s="5" t="str">
-        <v>EZDYH0000122</v>
+        <v>EFAZZ2400188</v>
       </c>
       <c r="B211" s="5" t="str">
         <v>800G PSM8</v>
       </c>
       <c r="C211" s="6" t="str">
-        <v>#12</v>
+        <v>#03</v>
       </c>
       <c r="D211" s="5" t="str">
         <v>TRX FA</v>
@@ -3479,153 +3479,153 @@
     </row>
     <row r="212">
       <c r="A212" s="5" t="str">
-        <v/>
+        <v>EFAZZ2400189</v>
       </c>
       <c r="B212" s="5" t="str">
-        <v/>
+        <v>800G PSM8</v>
       </c>
       <c r="C212" s="6" t="str">
-        <v/>
+        <v>#04</v>
       </c>
       <c r="D212" s="5" t="str">
-        <v/>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="5" t="str">
-        <v>EQPTZ2501092</v>
+        <v>EZDYH2400070</v>
       </c>
       <c r="B213" s="5" t="str">
         <v>800G PSM8</v>
       </c>
       <c r="C213" s="6" t="str">
-        <v>#02</v>
+        <v>#05</v>
       </c>
       <c r="D213" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="5" t="str">
-        <v>EZDYH2400050</v>
+        <v>EFAZZ2400187</v>
       </c>
       <c r="B214" s="5" t="str">
         <v>800G PSM8</v>
       </c>
       <c r="C214" s="6" t="str">
-        <v>#03</v>
+        <v>#06</v>
       </c>
       <c r="D214" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="5" t="str">
-        <v>EZDYH2400052</v>
+        <v>EFAZZ0001861</v>
       </c>
       <c r="B215" s="5" t="str">
         <v>800G PSM8</v>
       </c>
       <c r="C215" s="6" t="str">
-        <v>#04</v>
+        <v>#07</v>
       </c>
       <c r="D215" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="5" t="str">
-        <v>EZDYH2400055</v>
+        <v>EZDYH0000126</v>
       </c>
       <c r="B216" s="5" t="str">
         <v>800G PSM8</v>
       </c>
       <c r="C216" s="6" t="str">
-        <v>#05</v>
+        <v>#08</v>
       </c>
       <c r="D216" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="5" t="str">
-        <v>EQPTZ2500006</v>
+        <v>EFAQA0001820</v>
       </c>
       <c r="B217" s="5" t="str">
         <v>800G PSM8</v>
       </c>
       <c r="C217" s="6" t="str">
-        <v>#06</v>
+        <v>#10</v>
       </c>
       <c r="D217" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="5" t="str">
-        <v>EQPTZ2500001</v>
+        <v>EZDYH0000119</v>
       </c>
       <c r="B218" s="5" t="str">
         <v>800G PSM8</v>
       </c>
       <c r="C218" s="6" t="str">
-        <v>#07</v>
+        <v>#10</v>
       </c>
       <c r="D218" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="5" t="str">
-        <v>EQPTZ2500002</v>
+        <v>EFAZZ0001768</v>
       </c>
       <c r="B219" s="5" t="str">
         <v>800G PSM8</v>
       </c>
       <c r="C219" s="6" t="str">
-        <v>#08</v>
+        <v>#11</v>
       </c>
       <c r="D219" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="5" t="str">
-        <v>EZDYH2400057</v>
+        <v>EZDYH0000122</v>
       </c>
       <c r="B220" s="5" t="str">
         <v>800G PSM8</v>
       </c>
       <c r="C220" s="6" t="str">
-        <v>#09</v>
+        <v>#12</v>
       </c>
       <c r="D220" s="5" t="str">
-        <v>TX AA</v>
+        <v>TRX FA</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="5" t="str">
-        <v>EQPTZ2501099</v>
+        <v/>
       </c>
       <c r="B221" s="5" t="str">
-        <v>800G PSM8</v>
+        <v/>
       </c>
       <c r="C221" s="6" t="str">
-        <v>#10</v>
+        <v/>
       </c>
       <c r="D221" s="5" t="str">
-        <v>TX AA</v>
+        <v/>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="5" t="str">
-        <v>EQPTZ2501097</v>
+        <v>EQPTZ2501092</v>
       </c>
       <c r="B222" s="5" t="str">
         <v>800G PSM8</v>
       </c>
       <c r="C222" s="6" t="str">
-        <v>#12</v>
+        <v>#02</v>
       </c>
       <c r="D222" s="5" t="str">
         <v>TX AA</v>
@@ -3633,13 +3633,13 @@
     </row>
     <row r="223">
       <c r="A223" s="5" t="str">
-        <v>EQPTZ2501094</v>
+        <v>EZDYH2400050</v>
       </c>
       <c r="B223" s="5" t="str">
         <v>800G PSM8</v>
       </c>
       <c r="C223" s="6" t="str">
-        <v>#13</v>
+        <v>#03</v>
       </c>
       <c r="D223" s="5" t="str">
         <v>TX AA</v>
@@ -3647,114 +3647,114 @@
     </row>
     <row r="224">
       <c r="A224" s="5" t="str">
-        <v/>
+        <v>EZDYH2400052</v>
       </c>
       <c r="B224" s="5" t="str">
-        <v/>
+        <v>800G PSM8</v>
       </c>
       <c r="C224" s="6" t="str">
-        <v/>
+        <v>#04</v>
       </c>
       <c r="D224" s="5" t="str">
-        <v/>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="5" t="str">
-        <v>EFAZZ0001033</v>
+        <v>EQPTZ2500006</v>
       </c>
       <c r="B225" s="5" t="str">
-        <v>QDD AOC GEN3</v>
+        <v>800G PSM8</v>
       </c>
       <c r="C225" s="6" t="str">
-        <v>#00</v>
+        <v>#06</v>
       </c>
       <c r="D225" s="5" t="str">
-        <v>MM AA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="5" t="str">
-        <v/>
+        <v>EQPTZ2500001</v>
       </c>
       <c r="B226" s="5" t="str">
-        <v/>
+        <v>800G PSM8</v>
       </c>
       <c r="C226" s="6" t="str">
-        <v/>
+        <v>#07</v>
       </c>
       <c r="D226" s="5" t="str">
-        <v/>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="5" t="str">
-        <v>EFAZZ0000467</v>
+        <v>EQPTZ2500002</v>
       </c>
       <c r="B227" s="5" t="str">
-        <v>SR8 GEN2</v>
+        <v>800G PSM8</v>
       </c>
       <c r="C227" s="6" t="str">
-        <v>#04</v>
+        <v>#08</v>
       </c>
       <c r="D227" s="5" t="str">
-        <v>MM AA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="5" t="str">
-        <v>EFAZZ0000221</v>
+        <v>EZDYH2400057</v>
       </c>
       <c r="B228" s="5" t="str">
-        <v>SR8 GEN2</v>
+        <v>800G PSM8</v>
       </c>
       <c r="C228" s="6" t="str">
-        <v>#05</v>
+        <v>#09</v>
       </c>
       <c r="D228" s="5" t="str">
-        <v>MM AA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="5" t="str">
-        <v>EFAZZ0000155</v>
+        <v>EQPTZ2501099</v>
       </c>
       <c r="B229" s="5" t="str">
-        <v>SR8 GEN2</v>
+        <v>800G PSM8</v>
       </c>
       <c r="C229" s="6" t="str">
-        <v>#06</v>
+        <v>#10</v>
       </c>
       <c r="D229" s="5" t="str">
-        <v>MM AA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="5" t="str">
-        <v>EFAZZ0000153</v>
+        <v>EQPTZ2501097</v>
       </c>
       <c r="B230" s="5" t="str">
-        <v>SR8 GEN2</v>
+        <v>800G PSM8</v>
       </c>
       <c r="C230" s="6" t="str">
-        <v>#07</v>
+        <v>#12</v>
       </c>
       <c r="D230" s="5" t="str">
-        <v>MM AA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="5" t="str">
-        <v>EFAZZ0000400</v>
+        <v>EQPTZ2501094</v>
       </c>
       <c r="B231" s="5" t="str">
-        <v>SR8 GEN2</v>
+        <v>800G PSM8</v>
       </c>
       <c r="C231" s="6" t="str">
-        <v>#08</v>
+        <v>#13</v>
       </c>
       <c r="D231" s="5" t="str">
-        <v>MM AA</v>
+        <v>TX AA</v>
       </c>
     </row>
     <row r="232">
@@ -3773,21 +3773,133 @@
     </row>
     <row r="233">
       <c r="A233" s="5" t="str">
+        <v>EFAZZ0001033</v>
+      </c>
+      <c r="B233" s="5" t="str">
+        <v>QDD AOC GEN3</v>
+      </c>
+      <c r="C233" s="6" t="str">
+        <v>#00</v>
+      </c>
+      <c r="D233" s="5" t="str">
+        <v>MM AA</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="5" t="str">
+        <v/>
+      </c>
+      <c r="B234" s="5" t="str">
+        <v/>
+      </c>
+      <c r="C234" s="6" t="str">
+        <v/>
+      </c>
+      <c r="D234" s="5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="5" t="str">
+        <v>EFAZZ0000467</v>
+      </c>
+      <c r="B235" s="5" t="str">
+        <v>SR8 GEN2</v>
+      </c>
+      <c r="C235" s="6" t="str">
+        <v>#04</v>
+      </c>
+      <c r="D235" s="5" t="str">
+        <v>MM AA</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="5" t="str">
+        <v>EFAZZ0000221</v>
+      </c>
+      <c r="B236" s="5" t="str">
+        <v>SR8 GEN2</v>
+      </c>
+      <c r="C236" s="6" t="str">
+        <v>#05</v>
+      </c>
+      <c r="D236" s="5" t="str">
+        <v>MM AA</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="5" t="str">
+        <v>EFAZZ0000155</v>
+      </c>
+      <c r="B237" s="5" t="str">
+        <v>SR8 GEN2</v>
+      </c>
+      <c r="C237" s="6" t="str">
+        <v>#06</v>
+      </c>
+      <c r="D237" s="5" t="str">
+        <v>MM AA</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="5" t="str">
+        <v>EFAZZ0000153</v>
+      </c>
+      <c r="B238" s="5" t="str">
+        <v>SR8 GEN2</v>
+      </c>
+      <c r="C238" s="6" t="str">
+        <v>#07</v>
+      </c>
+      <c r="D238" s="5" t="str">
+        <v>MM AA</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="5" t="str">
+        <v>EFAZZ0000400</v>
+      </c>
+      <c r="B239" s="5" t="str">
+        <v>SR8 GEN2</v>
+      </c>
+      <c r="C239" s="6" t="str">
+        <v>#08</v>
+      </c>
+      <c r="D239" s="5" t="str">
+        <v>MM AA</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="5" t="str">
+        <v/>
+      </c>
+      <c r="B240" s="5" t="str">
+        <v/>
+      </c>
+      <c r="C240" s="6" t="str">
+        <v/>
+      </c>
+      <c r="D240" s="5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="5" t="str">
         <v>EFAZZ0000841</v>
       </c>
-      <c r="B233" s="5" t="str">
+      <c r="B241" s="5" t="str">
         <v>100G  DR1</v>
       </c>
-      <c r="C233" s="6" t="str">
+      <c r="C241" s="6" t="str">
         <v>#01</v>
       </c>
-      <c r="D233" s="5" t="str">
+      <c r="D241" s="5" t="str">
         <v>TX AA</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D233"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D241"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>